<commit_message>
add continuous screens, clustering and a DIABLO panel to the integration stage
</commit_message>
<xml_diff>
--- a/04_Modules/02_Contrasts/c_data/02_contrasts.xlsx
+++ b/04_Modules/02_Contrasts/c_data/02_contrasts.xlsx
@@ -184,30 +184,30 @@
     <t>outcome</t>
   </si>
   <si>
+    <t>pct_fcsa_mixed</t>
+  </si>
+  <si>
+    <t>pct_fcsa_type1</t>
+  </si>
+  <si>
+    <t>pct_fcsa_type2</t>
+  </si>
+  <si>
+    <t>pct_mcsa</t>
+  </si>
+  <si>
+    <t>pct_leg_press_1rm</t>
+  </si>
+  <si>
+    <t>pct_leg_ext_1rm</t>
+  </si>
+  <si>
     <t>comp_hypertrophy</t>
   </si>
   <si>
     <t>volume_load_total_kg</t>
   </si>
   <si>
-    <t>pct_fcsa_mixed</t>
-  </si>
-  <si>
-    <t>pct_fcsa_type1</t>
-  </si>
-  <si>
-    <t>pct_fcsa_type2</t>
-  </si>
-  <si>
-    <t>pct_mcsa</t>
-  </si>
-  <si>
-    <t>pct_leg_press_1rm</t>
-  </si>
-  <si>
-    <t>pct_leg_ext_1rm</t>
-  </si>
-  <si>
     <t>matrix</t>
   </si>
   <si>
@@ -343,7 +343,7 @@
     <t>modules</t>
   </si>
   <si>
-    <t>04_Network/01_Build_Modules/c_data/modules.rds</t>
+    <t>04_Modules/01_Build/c_data/modules.rds</t>
   </si>
   <si>
     <t>25cd43ced16098e9558525cfe4c1ef5e</t>
@@ -352,7 +352,7 @@
     <t>design</t>
   </si>
   <si>
-    <t>02_Differential_Expression/01_Design/c_data/design.rds</t>
+    <t>02_Proteins/01_Design/c_data/design.rds</t>
   </si>
   <si>
     <t>cbc0ed64f0e6b9a6f645c5aaad0ad907</t>
@@ -361,7 +361,7 @@
     <t>fit</t>
   </si>
   <si>
-    <t>02_Differential_Expression/02_Contrasts/c_data/fit.rds</t>
+    <t>02_Proteins/02_Contrasts/c_data/fit.rds</t>
   </si>
   <si>
     <t>76d83b782ba641782d378b9ae9391e38</t>
@@ -370,13 +370,13 @@
     <t>associate</t>
   </si>
   <si>
-    <t>02_Differential_Expression/04_Associate/c_data/associate.rds</t>
-  </si>
-  <si>
-    <t>e25e7c7d58c599c8dfb6b5fe8f919d4f</t>
-  </si>
-  <si>
-    <t>01_Preprocess/03_Quantification/c_data/DAList_limpa.rds</t>
+    <t>02_Proteins/04_Associate/c_data/associate.rds</t>
+  </si>
+  <si>
+    <t>3a76d72e831afb8502e14f9a9f644e34</t>
+  </si>
+  <si>
+    <t>01_Preprocess/03_Quantify/c_data/DAList_limpa.rds</t>
   </si>
   <si>
     <t>268362b9975bc00d3bc3b85b0f5736f7</t>
@@ -7716,13 +7716,13 @@
         <v>53</v>
       </c>
       <c r="C2">
-        <v>222</v>
+        <v>280</v>
       </c>
       <c r="D2">
-        <v>-0.02306426939200673</v>
+        <v>0.001278680975415096</v>
       </c>
       <c r="E2">
-        <v>0.7325350155698254</v>
+        <v>0.9830057716889404</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -7733,13 +7733,13 @@
         <v>54</v>
       </c>
       <c r="C3">
-        <v>222</v>
+        <v>280</v>
       </c>
       <c r="D3">
-        <v>0.4605067459891204</v>
+        <v>-0.08466514116736093</v>
       </c>
       <c r="E3">
-        <v>4.719153074944464E-13</v>
+        <v>0.1576794817468842</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -7750,13 +7750,13 @@
         <v>55</v>
       </c>
       <c r="C4">
-        <v>222</v>
+        <v>280</v>
       </c>
       <c r="D4">
-        <v>0.03433969735954086</v>
+        <v>-0.001386388195543575</v>
       </c>
       <c r="E4">
-        <v>0.6108141212991841</v>
+        <v>0.981574538997807</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -7767,13 +7767,13 @@
         <v>56</v>
       </c>
       <c r="C5">
-        <v>222</v>
+        <v>280</v>
       </c>
       <c r="D5">
-        <v>-0.06010990400476721</v>
+        <v>-0.08514669167336175</v>
       </c>
       <c r="E5">
-        <v>0.3727319326658359</v>
+        <v>0.1553212050183375</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -7784,13 +7784,13 @@
         <v>57</v>
       </c>
       <c r="C6">
-        <v>222</v>
+        <v>280</v>
       </c>
       <c r="D6">
-        <v>0.03889868591817405</v>
+        <v>-0.2877192890846091</v>
       </c>
       <c r="E6">
-        <v>0.5642612190972645</v>
+        <v>9.737846509354006E-07</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -7801,13 +7801,13 @@
         <v>58</v>
       </c>
       <c r="C7">
-        <v>222</v>
+        <v>280</v>
       </c>
       <c r="D7">
-        <v>-0.09020557356421076</v>
+        <v>0.06078533937158222</v>
       </c>
       <c r="E7">
-        <v>0.1805130265716584</v>
+        <v>0.310811544402154</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -7818,13 +7818,13 @@
         <v>59</v>
       </c>
       <c r="C8">
-        <v>222</v>
+        <v>280</v>
       </c>
       <c r="D8">
-        <v>-0.2849313643886531</v>
+        <v>-0.04278160232049547</v>
       </c>
       <c r="E8">
-        <v>1.624320223717274E-05</v>
+        <v>0.4758474915575154</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -7835,285 +7835,285 @@
         <v>60</v>
       </c>
       <c r="C9">
-        <v>222</v>
+        <v>280</v>
       </c>
       <c r="D9">
-        <v>0.09821176400051655</v>
+        <v>0.4589440394035665</v>
       </c>
       <c r="E9">
-        <v>0.1446779961485876</v>
+        <v>5.422129339069446E-16</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B10" t="s">
         <v>53</v>
       </c>
       <c r="C10">
-        <v>74</v>
+        <v>156</v>
       </c>
       <c r="D10">
-        <v>-0.03216848476671245</v>
+        <v>-0.2080044009744871</v>
       </c>
       <c r="E10">
-        <v>0.7855581718938981</v>
+        <v>0.009170192260385724</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
         <v>54</v>
       </c>
       <c r="C11">
-        <v>74</v>
+        <v>156</v>
       </c>
       <c r="D11">
-        <v>0.05539304658902438</v>
+        <v>-0.194957375317881</v>
       </c>
       <c r="E11">
-        <v>0.6392435109601282</v>
+        <v>0.01473275550764315</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
         <v>55</v>
       </c>
       <c r="C12">
-        <v>74</v>
+        <v>156</v>
       </c>
       <c r="D12">
-        <v>-0.06004280336183453</v>
+        <v>-0.1984216054496494</v>
       </c>
       <c r="E12">
-        <v>0.6113318819510833</v>
+        <v>0.01302467079098273</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s">
         <v>56</v>
       </c>
       <c r="C13">
-        <v>74</v>
+        <v>156</v>
       </c>
       <c r="D13">
-        <v>-0.1567024369427374</v>
+        <v>-0.1116874189988144</v>
       </c>
       <c r="E13">
-        <v>0.1824302214753427</v>
+        <v>0.1651055934629281</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B14" t="s">
         <v>57</v>
       </c>
       <c r="C14">
-        <v>74</v>
+        <v>156</v>
       </c>
       <c r="D14">
-        <v>-0.1004628435864579</v>
+        <v>-0.1316368666247795</v>
       </c>
       <c r="E14">
-        <v>0.3944036158602227</v>
+        <v>0.1014097900121884</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B15" t="s">
         <v>58</v>
       </c>
       <c r="C15">
-        <v>74</v>
+        <v>156</v>
       </c>
       <c r="D15">
-        <v>0.03220025214910374</v>
+        <v>0.03210425873388534</v>
       </c>
       <c r="E15">
-        <v>0.7853514784638443</v>
+        <v>0.6907335727921815</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B16" t="s">
         <v>59</v>
       </c>
       <c r="C16">
-        <v>74</v>
+        <v>156</v>
       </c>
       <c r="D16">
-        <v>-0.1567570376866445</v>
+        <v>-0.2296448570879741</v>
       </c>
       <c r="E16">
-        <v>0.1822759623132098</v>
+        <v>0.003928593841230781</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B17" t="s">
         <v>60</v>
       </c>
       <c r="C17">
-        <v>76</v>
+        <v>156</v>
       </c>
       <c r="D17">
-        <v>-0.3119996271109929</v>
+        <v>-0.05487058440002986</v>
       </c>
       <c r="E17">
-        <v>0.006074721521556788</v>
+        <v>0.4962927708649373</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B18" t="s">
         <v>53</v>
       </c>
       <c r="C18">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="D18">
-        <v>0.04347826086956522</v>
+        <v>0.004973538262603986</v>
       </c>
       <c r="E18">
-        <v>0.8438440075057314</v>
+        <v>0.9612348107509303</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B19" t="s">
         <v>54</v>
       </c>
       <c r="C19">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="D19">
-        <v>0.02075098814229249</v>
+        <v>-0.1140793035640538</v>
       </c>
       <c r="E19">
-        <v>0.9251264681656184</v>
+        <v>0.2633562719515128</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B20" t="s">
         <v>55</v>
       </c>
       <c r="C20">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="D20">
-        <v>0.09589719411850228</v>
+        <v>0.002984056354577352</v>
       </c>
       <c r="E20">
-        <v>0.6633701092843294</v>
+        <v>0.976735637264005</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B21" t="s">
         <v>56</v>
       </c>
       <c r="C21">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="D21">
-        <v>0.07808253265306767</v>
+        <v>0.0821522986360947</v>
       </c>
       <c r="E21">
-        <v>0.7232421082790783</v>
+        <v>0.4212859841648171</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B22" t="s">
         <v>57</v>
       </c>
       <c r="C22">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="D22">
-        <v>0.05782060962284125</v>
+        <v>-0.2585305993617095</v>
       </c>
       <c r="E22">
-        <v>0.7932806174098807</v>
+        <v>0.0101598669825922</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B23" t="s">
         <v>58</v>
       </c>
       <c r="C23">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="D23">
-        <v>-0.3389328063241107</v>
+        <v>-0.318535602312739</v>
       </c>
       <c r="E23">
-        <v>0.1136358510217293</v>
+        <v>0.001390676775111775</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B24" t="s">
         <v>59</v>
       </c>
       <c r="C24">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="D24">
-        <v>-0.02075098814229249</v>
+        <v>0.06385604112936341</v>
       </c>
       <c r="E24">
-        <v>0.9251264681656184</v>
+        <v>0.5321877961480079</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B25" t="s">
         <v>60</v>
       </c>
       <c r="C25">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="D25">
-        <v>0.3380281793335335</v>
+        <v>0.1040506298534691</v>
       </c>
       <c r="E25">
-        <v>0.1146646276081478</v>
+        <v>0.307916653381549</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -8124,13 +8124,13 @@
         <v>53</v>
       </c>
       <c r="C26">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="D26">
-        <v>0.1241739953278322</v>
+        <v>0.08274494404380596</v>
       </c>
       <c r="E26">
-        <v>0.1131533641811331</v>
+        <v>0.2589350005834374</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -8141,13 +8141,13 @@
         <v>54</v>
       </c>
       <c r="C27">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="D27">
-        <v>0.07602921518012778</v>
+        <v>0.02551024557965708</v>
       </c>
       <c r="E27">
-        <v>0.3332426223819152</v>
+        <v>0.7282137447705015</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -8158,13 +8158,13 @@
         <v>55</v>
       </c>
       <c r="C28">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="D28">
-        <v>0.08068438218338704</v>
+        <v>0.1142977895865505</v>
       </c>
       <c r="E28">
-        <v>0.3044032716373696</v>
+        <v>0.1183249542675263</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -8175,13 +8175,13 @@
         <v>56</v>
       </c>
       <c r="C29">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="D29">
-        <v>0.01825183920695871</v>
+        <v>0.1028546815936563</v>
       </c>
       <c r="E29">
-        <v>0.8165620166091404</v>
+        <v>0.1601418256046117</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -8192,13 +8192,13 @@
         <v>57</v>
       </c>
       <c r="C30">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="D30">
-        <v>0.1138334147063986</v>
+        <v>0.1133476410389972</v>
       </c>
       <c r="E30">
-        <v>0.1466822400445908</v>
+        <v>0.1214358359723519</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -8209,13 +8209,13 @@
         <v>58</v>
       </c>
       <c r="C31">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="D31">
-        <v>0.09309757064307542</v>
+        <v>0.05261584680018814</v>
       </c>
       <c r="E31">
-        <v>0.235745366682088</v>
+        <v>0.4733015476481311</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -8226,13 +8226,13 @@
         <v>59</v>
       </c>
       <c r="C32">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="D32">
-        <v>0.0729544519812225</v>
+        <v>0.1284275255111432</v>
       </c>
       <c r="E32">
-        <v>0.353218493346406</v>
+        <v>0.07901223425738818</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -8243,421 +8243,421 @@
         <v>60</v>
       </c>
       <c r="C33">
-        <v>166</v>
+        <v>188</v>
       </c>
       <c r="D33">
-        <v>0.05035513049050835</v>
+        <v>0.08239822146661141</v>
       </c>
       <c r="E33">
-        <v>0.5193893570819044</v>
+        <v>0.2609429170555813</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B34" t="s">
         <v>53</v>
       </c>
       <c r="C34">
-        <v>327</v>
+        <v>47</v>
       </c>
       <c r="D34">
-        <v>0.01712061669473723</v>
+        <v>0.2628885408769737</v>
       </c>
       <c r="E34">
-        <v>0.7577539494070206</v>
+        <v>0.07421415768461617</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B35" t="s">
         <v>54</v>
       </c>
       <c r="C35">
-        <v>327</v>
+        <v>47</v>
       </c>
       <c r="D35">
-        <v>-0.1027235855880866</v>
+        <v>0.2549008307598753</v>
       </c>
       <c r="E35">
-        <v>0.06354444657871169</v>
+        <v>0.08378279542051072</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B36" t="s">
         <v>55</v>
       </c>
       <c r="C36">
-        <v>327</v>
+        <v>47</v>
       </c>
       <c r="D36">
-        <v>0.02804910412459168</v>
+        <v>0.2060830359565684</v>
       </c>
       <c r="E36">
-        <v>0.6132968480494257</v>
+        <v>0.1646019127573573</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B37" t="s">
         <v>56</v>
       </c>
       <c r="C37">
-        <v>327</v>
+        <v>47</v>
       </c>
       <c r="D37">
-        <v>0.09341936915122698</v>
+        <v>-0.2593385006355806</v>
       </c>
       <c r="E37">
-        <v>0.09169247851663812</v>
+        <v>0.07835438296803228</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B38" t="s">
         <v>57</v>
       </c>
       <c r="C38">
-        <v>327</v>
+        <v>47</v>
       </c>
       <c r="D38">
-        <v>0.03690320391503422</v>
+        <v>-0.05603585484157227</v>
       </c>
       <c r="E38">
-        <v>0.5060524336111755</v>
+        <v>0.7083209398227269</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B39" t="s">
         <v>58</v>
       </c>
       <c r="C39">
-        <v>327</v>
+        <v>47</v>
       </c>
       <c r="D39">
-        <v>-0.04434872960422367</v>
+        <v>0.2672603232859874</v>
       </c>
       <c r="E39">
-        <v>0.4241242110370997</v>
+        <v>0.0693550812736158</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B40" t="s">
         <v>59</v>
       </c>
       <c r="C40">
-        <v>327</v>
+        <v>47</v>
       </c>
       <c r="D40">
-        <v>0.274573760320912</v>
+        <v>0.1272227870500093</v>
       </c>
       <c r="E40">
-        <v>4.573244598716264E-07</v>
+        <v>0.3941143106656196</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B41" t="s">
         <v>60</v>
       </c>
       <c r="C41">
-        <v>335</v>
+        <v>47</v>
       </c>
       <c r="D41">
-        <v>-0.1340633108898234</v>
+        <v>0.1750621783908307</v>
       </c>
       <c r="E41">
-        <v>0.0140616330733876</v>
+        <v>0.2392099813052794</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B42" t="s">
         <v>53</v>
       </c>
       <c r="C42">
-        <v>75</v>
+        <v>402</v>
       </c>
       <c r="D42">
-        <v>0.09050301596534154</v>
+        <v>-0.002331844886578274</v>
       </c>
       <c r="E42">
-        <v>0.4399951368941133</v>
+        <v>0.9628257976104719</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B43" t="s">
         <v>54</v>
       </c>
       <c r="C43">
-        <v>75</v>
+        <v>402</v>
       </c>
       <c r="D43">
-        <v>0.05287791295900515</v>
+        <v>0.07052477334509397</v>
       </c>
       <c r="E43">
-        <v>0.6523066095047463</v>
+        <v>0.1581349388221162</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B44" t="s">
         <v>55</v>
       </c>
       <c r="C44">
-        <v>75</v>
+        <v>402</v>
       </c>
       <c r="D44">
-        <v>-0.02587611050698982</v>
+        <v>0.003718490678062852</v>
       </c>
       <c r="E44">
-        <v>0.8255855784666662</v>
+        <v>0.940752895715558</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B45" t="s">
         <v>56</v>
       </c>
       <c r="C45">
-        <v>75</v>
+        <v>402</v>
       </c>
       <c r="D45">
-        <v>-0.03132446142737305</v>
+        <v>-0.0146120127621921</v>
       </c>
       <c r="E45">
-        <v>0.7896332507063825</v>
+        <v>0.7702306136125863</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B46" t="s">
         <v>57</v>
       </c>
       <c r="C46">
-        <v>75</v>
+        <v>402</v>
       </c>
       <c r="D46">
-        <v>-0.04748627211653463</v>
+        <v>0.3170131801146648</v>
       </c>
       <c r="E46">
-        <v>0.6857977863783312</v>
+        <v>7.777949429944137E-11</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B47" t="s">
         <v>58</v>
       </c>
       <c r="C47">
-        <v>75</v>
+        <v>402</v>
       </c>
       <c r="D47">
-        <v>0.1085306611936559</v>
+        <v>-0.1016640257348501</v>
       </c>
       <c r="E47">
-        <v>0.3540001656188557</v>
+        <v>0.04162085766040832</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B48" t="s">
         <v>59</v>
       </c>
       <c r="C48">
-        <v>75</v>
+        <v>402</v>
       </c>
       <c r="D48">
-        <v>0.03765479082572955</v>
+        <v>-0.0002633214955349744</v>
       </c>
       <c r="E48">
-        <v>0.7484099538955648</v>
+        <v>0.9958006416270667</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B49" t="s">
         <v>60</v>
       </c>
       <c r="C49">
-        <v>77</v>
+        <v>402</v>
       </c>
       <c r="D49">
-        <v>0.02930099579163533</v>
+        <v>-0.1432751546504037</v>
       </c>
       <c r="E49">
-        <v>0.8002960145152074</v>
+        <v>0.003994725534693253</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B50" t="s">
         <v>53</v>
       </c>
       <c r="C50">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D50">
-        <v>-0.2669873132830539</v>
+        <v>-0.03673108473710941</v>
       </c>
       <c r="E50">
-        <v>0.003921679448737283</v>
+        <v>0.7085442493935078</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B51" t="s">
         <v>54</v>
       </c>
       <c r="C51">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D51">
-        <v>-0.01652791478895477</v>
+        <v>-0.05827581011252504</v>
       </c>
       <c r="E51">
-        <v>0.860829880537509</v>
+        <v>0.5529290026918783</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B52" t="s">
         <v>55</v>
       </c>
       <c r="C52">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D52">
-        <v>-0.2689195990605323</v>
+        <v>0.004428802845092846</v>
       </c>
       <c r="E52">
-        <v>0.003659993008050823</v>
+        <v>0.9640619653121232</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B53" t="s">
         <v>56</v>
       </c>
       <c r="C53">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D53">
-        <v>-0.282923057263757</v>
+        <v>0.1443820499907613</v>
       </c>
       <c r="E53">
-        <v>0.002186043469406961</v>
+        <v>0.1397754656276197</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B54" t="s">
         <v>57</v>
       </c>
       <c r="C54">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D54">
-        <v>-0.2348074149554265</v>
+        <v>0.1273350687254461</v>
       </c>
       <c r="E54">
-        <v>0.01153889035401647</v>
+        <v>0.1933432447773169</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B55" t="s">
         <v>58</v>
       </c>
       <c r="C55">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D55">
-        <v>-0.08248305371516511</v>
+        <v>0.02207934870497028</v>
       </c>
       <c r="E55">
-        <v>0.3808322536461833</v>
+        <v>0.8222493402571578</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B56" t="s">
         <v>59</v>
       </c>
       <c r="C56">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D56">
-        <v>-0.1862216716348315</v>
+        <v>0.1054331454904871</v>
       </c>
       <c r="E56">
-        <v>0.04629919408639283</v>
+        <v>0.2820922209703421</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B57" t="s">
         <v>60</v>
       </c>
       <c r="C57">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D57">
-        <v>0.0009627126408170587</v>
+        <v>0.03013561286867646</v>
       </c>
       <c r="E57">
-        <v>0.991852812802569</v>
+        <v>0.7591052300432984</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -8668,13 +8668,13 @@
         <v>53</v>
       </c>
       <c r="C58">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="D58">
-        <v>0.3791758416497666</v>
+        <v>0.2756678428095846</v>
       </c>
       <c r="E58">
-        <v>0.001313461780509801</v>
+        <v>0.01593987616710842</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -8685,13 +8685,13 @@
         <v>54</v>
       </c>
       <c r="C59">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="D59">
-        <v>0.05745761488595771</v>
+        <v>0.2224045187731568</v>
       </c>
       <c r="E59">
-        <v>0.6391073825170078</v>
+        <v>0.05348260261542722</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -8702,13 +8702,13 @@
         <v>55</v>
       </c>
       <c r="C60">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="D60">
-        <v>0.2329298929125028</v>
+        <v>0.3414934299148747</v>
       </c>
       <c r="E60">
-        <v>0.05409220481113665</v>
+        <v>0.002535702032154434</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -8719,13 +8719,13 @@
         <v>56</v>
       </c>
       <c r="C61">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="D61">
-        <v>0.2028135570716572</v>
+        <v>0.3984168335607683</v>
       </c>
       <c r="E61">
-        <v>0.09465504809613784</v>
+        <v>0.0003644855940593978</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -8736,13 +8736,13 @@
         <v>57</v>
       </c>
       <c r="C62">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="D62">
-        <v>0.3379558612437272</v>
+        <v>-0.2815873139184045</v>
       </c>
       <c r="E62">
-        <v>0.004510442731650399</v>
+        <v>0.01373114225023653</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -8753,13 +8753,13 @@
         <v>58</v>
       </c>
       <c r="C63">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="D63">
-        <v>0.1699748802868961</v>
+        <v>0.3914883149949989</v>
       </c>
       <c r="E63">
-        <v>0.1626220118188599</v>
+        <v>0.0004704529474062494</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -8770,13 +8770,13 @@
         <v>59</v>
       </c>
       <c r="C64">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="D64">
-        <v>-0.199360556235107</v>
+        <v>0.4218729740742834</v>
       </c>
       <c r="E64">
-        <v>0.1005296856186939</v>
+        <v>0.0001472575945894611</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -8787,13 +8787,13 @@
         <v>60</v>
       </c>
       <c r="C65">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="D65">
-        <v>0.3162548530359479</v>
+        <v>0.09970602520507162</v>
       </c>
       <c r="E65">
-        <v>0.00811281153046337</v>
+        <v>0.391472841743701</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -8804,13 +8804,13 @@
         <v>53</v>
       </c>
       <c r="C66">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="D66">
-        <v>0.02183898572773505</v>
+        <v>0.05525758091631758</v>
       </c>
       <c r="E66">
-        <v>0.8152051878846418</v>
+        <v>0.5182222508625256</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -8821,13 +8821,13 @@
         <v>54</v>
       </c>
       <c r="C67">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="D67">
-        <v>0.07423310019705484</v>
+        <v>0.01017558132290561</v>
       </c>
       <c r="E67">
-        <v>0.4263628172021501</v>
+        <v>0.9053640368703415</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -8838,13 +8838,13 @@
         <v>55</v>
       </c>
       <c r="C68">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="D68">
-        <v>0.04017114513171646</v>
+        <v>0.03576843035526707</v>
       </c>
       <c r="E68">
-        <v>0.6671768979670354</v>
+        <v>0.6759256896045802</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -8855,13 +8855,13 @@
         <v>56</v>
       </c>
       <c r="C69">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="D69">
-        <v>0.02998518169717364</v>
+        <v>-0.04524887901170432</v>
       </c>
       <c r="E69">
-        <v>0.7482640493240694</v>
+        <v>0.5968539822515151</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -8872,13 +8872,13 @@
         <v>57</v>
       </c>
       <c r="C70">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="D70">
-        <v>0.02410238928611024</v>
+        <v>0.1467400598239061</v>
       </c>
       <c r="E70">
-        <v>0.7964489280777034</v>
+        <v>0.08475100205294422</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -8889,13 +8889,13 @@
         <v>58</v>
       </c>
       <c r="C71">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="D71">
-        <v>-0.04762386480849672</v>
+        <v>-0.03113244765445469</v>
       </c>
       <c r="E71">
-        <v>0.6101288435139355</v>
+        <v>0.7159925400655913</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -8906,13 +8906,13 @@
         <v>59</v>
       </c>
       <c r="C72">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="D72">
-        <v>0.1561131875995904</v>
+        <v>0.02734672634585295</v>
       </c>
       <c r="E72">
-        <v>0.09279901004602864</v>
+        <v>0.7493007931423936</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -8923,13 +8923,13 @@
         <v>60</v>
       </c>
       <c r="C73">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="D73">
-        <v>-0.04143101487372124</v>
+        <v>0.07958082451800941</v>
       </c>
       <c r="E73">
-        <v>0.6573868383531769</v>
+        <v>0.3517245010259016</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -8940,13 +8940,13 @@
         <v>53</v>
       </c>
       <c r="C74">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="D74">
-        <v>-0.5206107112923827</v>
+        <v>-0.1881803705258812</v>
       </c>
       <c r="E74">
-        <v>0.005368407564390642</v>
+        <v>0.2002414075519774</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -8957,13 +8957,13 @@
         <v>54</v>
       </c>
       <c r="C75">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="D75">
-        <v>-0.1782661782661782</v>
+        <v>-0.1424693310476689</v>
       </c>
       <c r="E75">
-        <v>0.3736683508561941</v>
+        <v>0.3340555525615975</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -8974,13 +8974,13 @@
         <v>55</v>
       </c>
       <c r="C76">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="D76">
-        <v>-0.4693129989773561</v>
+        <v>-0.1679061962443517</v>
       </c>
       <c r="E76">
-        <v>0.01352471562948205</v>
+        <v>0.2539758600844356</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -8991,13 +8991,13 @@
         <v>56</v>
       </c>
       <c r="C77">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="D77">
-        <v>-0.3124141418030928</v>
+        <v>0.03180806605130926</v>
       </c>
       <c r="E77">
-        <v>0.1126161468092624</v>
+        <v>0.8300651497354899</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -9008,13 +9008,13 @@
         <v>57</v>
       </c>
       <c r="C78">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="D78">
-        <v>-0.5019081114803462</v>
+        <v>-0.4110734170228182</v>
       </c>
       <c r="E78">
-        <v>0.007641078533147146</v>
+        <v>0.003702750780723886</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -9025,13 +9025,13 @@
         <v>58</v>
       </c>
       <c r="C79">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="D79">
-        <v>-0.05799755799755799</v>
+        <v>0.09860723539159676</v>
       </c>
       <c r="E79">
-        <v>0.7738475387037593</v>
+        <v>0.5049058315901928</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -9042,13 +9042,13 @@
         <v>59</v>
       </c>
       <c r="C80">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="D80">
-        <v>-0.3837582093253012</v>
+        <v>-0.1703490603992162</v>
       </c>
       <c r="E80">
-        <v>0.04814176054174718</v>
+        <v>0.2470323885632009</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -9059,13 +9059,13 @@
         <v>60</v>
       </c>
       <c r="C81">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="D81">
-        <v>-0.06350944667199004</v>
+        <v>-0.0838716693170137</v>
       </c>
       <c r="E81">
-        <v>0.7481626714884575</v>
+        <v>0.5708752029002331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>